<commit_message>
AML (マウスレイヤー) を Ctrl / Shift / Win / Alt で解除する (#24)
ryo-aoki-pc/zmk-config-LisM#22 と同じ内容 (LisM 基準)。

- excluded-positions を D / K (&mo SCRL、12 / 17) だけにする。修飾キーの位置
  (A / - / Z / / / Win / Alt) を押すと AML が切れる
- MOUSE_MOVE の修飾キーの位置を &trans にする (BASE と同じ &mt / &kp。タップで文字、
  長押しで修飾キー)
- MOUSE_SCROLL の修飾キーはそのまま。修飾キーとクリック・ホイールを組み合わせるときは
  D / K を押してから修飾キーを押す (例: D → Z → F で Shift + クリック)
- excluded-positions を説明する補足コメントも直す
- KEYMAP.html / KEYMAP.xlsx を作り直す

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QFG6t92cGtjhGTDoN62Yvg
</commit_message>
<xml_diff>
--- a/KEYMAP.xlsx
+++ b/KEYMAP.xlsx
@@ -5054,7 +5054,7 @@
       <c r="B97" s="7" t="inlineStr">
         <is>
           <t>pos 10
-&amp;kp LCTRL</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
@@ -5109,7 +5109,7 @@
       <c r="L97" s="7" t="inlineStr">
         <is>
           <t>pos 19
-&amp;kp RCTRL</t>
+&amp;trans</t>
         </is>
       </c>
     </row>
@@ -5121,7 +5121,7 @@
       </c>
       <c r="B98" s="9" t="inlineStr">
         <is>
-          <t>LCtrl</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="C98" s="9" t="inlineStr"/>
@@ -5143,7 +5143,7 @@
       <c r="K98" s="9" t="inlineStr"/>
       <c r="L98" s="9" t="inlineStr">
         <is>
-          <t>RCtrl</t>
+          <t>▽</t>
         </is>
       </c>
     </row>
@@ -5156,7 +5156,7 @@
       <c r="B99" s="7" t="inlineStr">
         <is>
           <t>pos 20
-&amp;kp LEFT_SHIFT</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="C99" s="7" t="inlineStr">
@@ -5223,7 +5223,7 @@
       </c>
       <c r="B100" s="9" t="inlineStr">
         <is>
-          <t>LShift</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="C100" s="9" t="inlineStr"/>
@@ -5252,19 +5252,19 @@
       <c r="C101" s="7" t="inlineStr">
         <is>
           <t>pos 31
-&amp;kp RIGHT_SHIFT</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
         <is>
           <t>pos 32
-&amp;kp LEFT_WIN</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
         <is>
           <t>pos 33
-&amp;kp LEFT_ALT</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="F101" s="7" t="inlineStr">
@@ -5314,17 +5314,17 @@
       <c r="B102" s="9" t="inlineStr"/>
       <c r="C102" s="9" t="inlineStr">
         <is>
-          <t>RShift</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="D102" s="9" t="inlineStr">
         <is>
-          <t>LWin</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="E102" s="9" t="inlineStr">
         <is>
-          <t>LAlt</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="F102" s="9" t="inlineStr"/>
@@ -10344,7 +10344,7 @@
       <c r="B97" s="7" t="inlineStr">
         <is>
           <t>pos 10
-&amp;kp LCTRL</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
@@ -10399,7 +10399,7 @@
       <c r="L97" s="7" t="inlineStr">
         <is>
           <t>pos 19
-&amp;kp RCTRL</t>
+&amp;trans</t>
         </is>
       </c>
     </row>
@@ -10411,7 +10411,7 @@
       </c>
       <c r="B98" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp LCTRL</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="C98" s="9" t="inlineStr"/>
@@ -10433,7 +10433,7 @@
       <c r="K98" s="9" t="inlineStr"/>
       <c r="L98" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp RCTRL</t>
+          <t>▽</t>
         </is>
       </c>
     </row>
@@ -10446,7 +10446,7 @@
       <c r="B99" s="7" t="inlineStr">
         <is>
           <t>pos 20
-&amp;kp LEFT_SHIFT</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="C99" s="7" t="inlineStr">
@@ -10513,7 +10513,7 @@
       </c>
       <c r="B100" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp LEFT_SHIFT</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="C100" s="9" t="inlineStr"/>
@@ -10542,19 +10542,19 @@
       <c r="C101" s="7" t="inlineStr">
         <is>
           <t>pos 31
-&amp;kp RIGHT_SHIFT</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
         <is>
           <t>pos 32
-&amp;kp LEFT_WIN</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
         <is>
           <t>pos 33
-&amp;kp LEFT_ALT</t>
+&amp;trans</t>
         </is>
       </c>
       <c r="F101" s="7" t="inlineStr">
@@ -10604,17 +10604,17 @@
       <c r="B102" s="9" t="inlineStr"/>
       <c r="C102" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp RIGHT_SHIFT</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="D102" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp LEFT_WIN</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="E102" s="9" t="inlineStr">
         <is>
-          <t>&amp;kp LEFT_ALT</t>
+          <t>▽</t>
         </is>
       </c>
       <c r="F102" s="9" t="inlineStr"/>

</xml_diff>